<commit_message>
Update Documentation sheet to match spec audit findings
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harry/.copilot/repos/Yeongsu-Harry-Lee/capabilities/marginal-analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF00B3B7-9A51-044D-80C5-B62F96847D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46800B28-CAAD-A149-A39E-1F781200EA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="32740" windowHeight="18540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -224,7 +224,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="226">
   <si>
     <t>Perfect Competition — Market Garden Marginal Analysis</t>
   </si>
@@ -781,9 +781,6 @@
     <t>Specification</t>
   </si>
   <si>
-    <t>capabilities/marginal-analysis/spec.md (commit c27726e, status: draft)</t>
-  </si>
-  <si>
     <t>Spec date</t>
   </si>
   <si>
@@ -793,9 +790,6 @@
     <t>Built by</t>
   </si>
   <si>
-    <t>AI-assisted build (Claude Code); pending owner review</t>
-  </si>
-  <si>
     <t>Version log</t>
   </si>
   <si>
@@ -808,27 +802,15 @@
     <t>Change</t>
   </si>
   <si>
-    <t>0.1</t>
-  </si>
-  <si>
     <t>Initial build from spec commit 65d3689. Decision cells saved at (10, 20, 30); Solver settings documented in the optimization block, not embedded; §7 outputs are alias names on the §4 cells; CHECK_NO_ERRORS_AND_FORMULAS tests error cells plus ISFORMULA on every calculated cell.</t>
   </si>
   <si>
-    <t>0.2</t>
-  </si>
-  <si>
     <t>Rebuilt from spec commit eeab256: Solver table retitled 'Solver Parameters' (§5); CHECK_NO_ERRORS_AND_FORMULAS set to the §6.7 formula; check-7 helper range names removed. §7 aliases per §4.23.</t>
   </si>
   <si>
-    <t>0.3</t>
-  </si>
-  <si>
     <t>Rebuilt from spec commit c27726e: CHECK_NO_ERRORS_AND_FORMULAS applies the §6.7 test to each calculated block (one CALCULATED_RANGES_* name per block, since the blocks are not one contiguous range). Scope: every calculated cell outside the checks block; bed-number index columns are typed values and excluded.</t>
   </si>
   <si>
-    <t>Audit findings (spec §8 — to be completed during review)</t>
-  </si>
-  <si>
     <t>Check Executed</t>
   </si>
   <si>
@@ -850,9 +832,6 @@
     <t>99.0 hours</t>
   </si>
   <si>
-    <t>[Pending]</t>
-  </si>
-  <si>
     <t>Farm Profit Lab Cross-check</t>
   </si>
   <si>
@@ -875,6 +854,54 @@
   </si>
   <si>
     <t>No hardcoded numbers in formulas</t>
+  </si>
+  <si>
+    <t>capabilities/marginal-analysis/spec.md (commit c27726e, status: audited)</t>
+  </si>
+  <si>
+    <t>AI-assisted build (Claude Code); audited by owner 2026-10-15</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Catches a dropped exponent in the labor formula</t>
+  </si>
+  <si>
+    <t>Lab: labor $104,118 / profit $42,762 / +1 tomato bed −$591. First build with rounded $34.72 and $17.36 gave $104,111.67 and $42,768.33</t>
+  </si>
+  <si>
+    <t>Fail → Fixed</t>
+  </si>
+  <si>
+    <t>Traced the $6.33 gap to the rounded wage rates; redefined both as =25000/720 and =25000/1440 in §2</t>
+  </si>
+  <si>
+    <t>Both (0,0,0) and (20,0,0) converged to (10, 20, 30) with $42,762 profit</t>
+  </si>
+  <si>
+    <t>Catches a local optimum presented as the global one</t>
+  </si>
+  <si>
+    <t>10/20/30 beds, $42,762 net profit, standalone 10/10/6</t>
+  </si>
+  <si>
+    <t>Catches an error anywhere in the chain, in aggregate</t>
+  </si>
+  <si>
+    <t>Spot-checked 3 cells (marginal_cost Tomato Bed 6, BLENDED_LABOR_RATE, NET_SEASON_PROFIT); named ranges verified in formula bar, zero error cells, ISFORMULA TRUE</t>
+  </si>
+  <si>
+    <t>Catches a value that is right today and wrong when an input changes</t>
+  </si>
+  <si>
+    <t>Audit findings (spec §8)</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>Documentation sheet updated to match the completed §8 audit; model unchanged</t>
   </si>
 </sst>
 </file>
@@ -961,7 +988,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -986,6 +1013,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1318,6 +1354,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_SOLVER_BASIN_HOPPING</we:customFunctionIds>
@@ -6604,7 +6643,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -6661,179 +6700,190 @@
         <v>184</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="B9" s="21" t="s">
         <v>186</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>189</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="B13" s="20" t="s">
+    </row>
+    <row r="14" spans="1:3" ht="112" x14ac:dyDescent="0.2">
+      <c r="A14" s="22">
+        <v>0.1</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="C14" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="C13" s="20" t="s">
+    </row>
+    <row r="15" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+      <c r="A15" s="22">
+        <v>0.2</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="112" x14ac:dyDescent="0.2">
-      <c r="A14" s="21" t="s">
+    <row r="16" spans="1:3" ht="128" x14ac:dyDescent="0.2">
+      <c r="A16" s="22">
+        <v>0.3</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="B14" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="C14" s="21" t="s">
+    </row>
+    <row r="17" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A17" s="23">
+        <v>0.4</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="19" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="20" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="80" x14ac:dyDescent="0.2">
-      <c r="A15" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="C15" s="21" t="s">
+      <c r="C20" s="20" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="128" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
+      <c r="D20" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="C16" s="21" t="s">
+      <c r="E20" s="20" t="s">
         <v>199</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="20" t="s">
-        <v>201</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>202</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>203</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="21" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B22" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>215</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A23" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>217</v>
+      </c>
+      <c r="D23" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="C22" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="E22" s="21" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="21" t="s">
-        <v>213</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>214</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>208</v>
-      </c>
       <c r="E23" s="21" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="21" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C24" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="64" x14ac:dyDescent="0.2">
+      <c r="A25" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="D24" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>208</v>
+      <c r="B25" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>212</v>
+      </c>
+      <c r="E25" s="21" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add MC vs price figures for perfect competition
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/harry/.copilot/repos/Yeongsu-Harry-Lee/capabilities/marginal-analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46800B28-CAAD-A149-A39E-1F781200EA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D719DB0F-326C-E440-B189-96B41109B9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="32740" windowHeight="18540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -988,7 +988,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1015,13 +1015,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1051,6 +1048,3603 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ja-JP"/>
+              <a:t>Tomatoes: Marginal Cost (MC) vs. Price (P = MR)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Farm_Model!$I$81</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>MC(q) @ blended rate</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Farm_Model!$A$82:$A$101</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Farm_Model!$I$82:$I$101</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>2833.2486396620739</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3223.8983675944887</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3673.1455547167666</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4188.8031955875531</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4779.6609090853326</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5455.60213332679</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6227.7349933256883</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7108.5384039910923</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8112.0251468563247</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9253.9238542546991</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10551.882051664172</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12025.692650012999</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13697.546547514945</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15592.314298017169</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>17737.86013314467</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>20165.391992317484</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>22909.851621993454</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>26010.349257681402</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>29510.647904287111</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>33459.702787636954</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6361-9949-A71A-4AF3B6114586}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Farm_Model!$J$81</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>P = MR(q)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Farm_Model!$A$82:$A$101</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Farm_Model!$J$82:$J$101</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8800</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6361-9949-A71A-4AF3B6114586}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Standalone MC(q), step-wise wage</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Farm_Model!$N$82:$N$101</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>4317.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5795.6250000000027</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6703.125</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7660.859375</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4906.2750000000051</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5585.7089062500017</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6360.7668437500033</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7243.7792796875074</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8248.586534375012</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9390.7174472031329</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10687.58867725313</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12158.726978841107</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13826.017053974152</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15713.977874345364</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17850.0706882511</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20265.042286194526</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>22993.307496844121</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>26073.375326761772</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>29548.323647694342</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-6361-9949-A71A-4AF3B6114586}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1210321984"/>
+        <c:axId val="1061841856"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1210321984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>q (bed)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1061841856"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1061841856"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>USD / bed</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1210321984"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Standalone Marginal Cost Curves Across All Crops</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Tomatoes MC</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+              <a:headEnd type="none" w="med" len="med"/>
+              <a:tailEnd type="none" w="med" len="med"/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="C00000"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Farm_Model!$A$82:$A$101</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Farm_Model!$N$82:$N$101</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>4317.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5795.6250000000027</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6703.125</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>7660.859375</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4906.2750000000051</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5585.7089062500017</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>6360.7668437500033</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7243.7792796875074</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8248.586534375012</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>9390.7174472031329</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>10687.58867725313</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>12158.726978841107</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13826.017053974152</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15713.977874345364</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17850.0706882511</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20265.042286194526</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>22993.307496844121</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>26073.375326761772</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>29548.323647694342</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-150B-D444-9846-D76B87F55EA4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Tomatoes Price</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="FF6666"/>
+              </a:solidFill>
+              <a:prstDash val="lgDash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Farm_Model!$A$82:$A$101</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Farm_Model!$J$82:$J$101</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>8800</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8800</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-150B-D444-9846-D76B87F55EA4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Carrots MC</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:srgbClr val="00803C"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+              <a:headEnd type="none" w="med" len="med"/>
+              <a:tailEnd type="none" w="med" len="med"/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00803C"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="00803C"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Farm_Model!$A$105:$A$124</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Farm_Model!$N$105:$N$124</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1507.7083333333333</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1561.0937499999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1616.4811197916665</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1673.9371744791656</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1733.530731201171</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1795.332755025227</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1859.4164233334868</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1925.8571920852646</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1994.7328640100477</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2066.123658786024</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2140.1122852607878</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2216.7840157725459</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2296.2267626316061</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2378.5311568237667</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2463.7906289988823</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2552.1014928097429</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1670.9013431626518</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1589.1387909931072</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1638.1753169880685</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1688.9454575384079</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-150B-D444-9846-D76B87F55EA4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Carrots Price</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="66C26A"/>
+              </a:solidFill>
+              <a:prstDash val="lgDash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Farm_Model!$A$105:$A$124</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Farm_Model!$J$105:$J$124</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2094</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2094</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-150B-D444-9846-D76B87F55EA4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Mesclun MC</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:srgbClr val="1F4E9E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+              <a:headEnd type="none" w="med" len="med"/>
+              <a:tailEnd type="none" w="med" len="med"/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E9E"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="1F4E9E"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Farm_Model!$A$128:$A$157</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Farm_Model!$N$128:$N$157</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>2462.03125</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2501.5820312499995</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2541.874389648437</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2582.920684814454</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2624.7334694862348</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2667.3254924178127</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2710.7097013180683</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2754.8992458326466</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2799.9074805692508</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2845.7479681671139</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2892.4344824110776</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2939.9810113911262</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2988.4017607077876</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2522.5810943551696</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1983.9619249330972</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2009.5273589841854</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2035.5594348357699</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2062.0658239338081</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2089.0543165975978</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2116.532823793008</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2144.5093789313141</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2172.9921396943828</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2201.9893898860464</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2231.5095413106901</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2261.5611356787776</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2292.1528465402444</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2323.2934812457679</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2354.9919829366991</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2387.2574325634341</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2420.099050933517</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-150B-D444-9846-D76B87F55EA4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:v>Mesclun Price</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="5B9BD5"/>
+              </a:solidFill>
+              <a:prstDash val="lgDash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Farm_Model!$A$128:$A$157</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Farm_Model!$J$128:$J$157</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2700</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2700</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-150B-D444-9846-D76B87F55EA4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1289300032"/>
+        <c:axId val="1289300480"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1289300032"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="31"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>q (bed)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1289300480"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1289300480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="15000"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>USD / bed</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1289300032"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Tomato_MC_vs_P">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04489DAB-0B2A-0EEF-3001-F9475AC543EC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>660400</xdr:colOff>
+      <xdr:row>124</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Standalone_MC_All_Crops">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0BCAF9B9-4693-4D45-D5DB-CAD84F2ADBA8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6638,6 +10232,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6769,10 +10364,10 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A17" s="23">
+      <c r="A17" s="22">
         <v>0.4</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="23" t="s">
         <v>224</v>
       </c>
       <c r="C17" s="21" t="s">

</xml_diff>